<commit_message>
Update controlled Minfin source latest registry
</commit_message>
<xml_diff>
--- a/data/raw/minfin/ofz_auction_results/latest/INTERNET_Auction_Results_rus_2026_latest.xlsx
+++ b/data/raw/minfin/ofz_auction_results/latest/INTERNET_Auction_Results_rus_2026_latest.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Лист1!$A$3:$O$69</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Лист1!$A$3:$O$71</definedName>
   </definedNames>
   <calcPr calcId="162913" calcMode="manual"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="47">
   <si>
     <t>По состоянию на</t>
   </si>
@@ -750,7 +750,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O71"/>
+  <dimension ref="A1:O73"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" style="1" customWidth="1"/>
@@ -780,7 +780,7 @@
         <v>0</v>
       </c>
       <c r="O3" s="5">
-        <v>46184</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="4" spans="1:15" ht="23.65" customHeight="1" x14ac:dyDescent="0.25">
@@ -3694,73 +3694,167 @@
       </c>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A68" s="10" t="s">
+      <c r="A68" s="10">
+        <v>46190</v>
+      </c>
+      <c r="B68" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C68" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="D68" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E68" s="10">
+        <v>48864</v>
+      </c>
+      <c r="F68" s="12">
+        <v>2674</v>
+      </c>
+      <c r="G68" s="13">
+        <v>297871.94299999997</v>
+      </c>
+      <c r="H68" s="14">
+        <v>91.740299999999991</v>
+      </c>
+      <c r="I68" s="14">
+        <v>91.788700000000006</v>
+      </c>
+      <c r="J68" s="15">
+        <v>14.860000000000001</v>
+      </c>
+      <c r="K68" s="15">
+        <v>14.85</v>
+      </c>
+      <c r="L68" s="13">
+        <v>124302.072</v>
+      </c>
+      <c r="M68" s="13">
+        <v>97767.57</v>
+      </c>
+      <c r="N68" s="13">
+        <v>91648.000480319999</v>
+      </c>
+      <c r="O68" s="16">
+        <v>0.78653210221628489</v>
+      </c>
+    </row>
+    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A69" s="10">
+        <v>46190</v>
+      </c>
+      <c r="B69" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C69" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="D69" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E69" s="10">
+        <v>51412</v>
+      </c>
+      <c r="F69" s="12">
+        <v>5222</v>
+      </c>
+      <c r="G69" s="13">
+        <v>343003.96799999999</v>
+      </c>
+      <c r="H69" s="14">
+        <v>91.43</v>
+      </c>
+      <c r="I69" s="14">
+        <v>91.448499999999996</v>
+      </c>
+      <c r="J69" s="15">
+        <v>14.940000000000001</v>
+      </c>
+      <c r="K69" s="15">
+        <v>14.940000000000001</v>
+      </c>
+      <c r="L69" s="13">
+        <v>54095.309000000001</v>
+      </c>
+      <c r="M69" s="13">
+        <v>22277.206999999999</v>
+      </c>
+      <c r="N69" s="13">
+        <v>20824.397864499999</v>
+      </c>
+      <c r="O69" s="16">
+        <v>0.41181402624024199</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A70" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B68" s="10" t="s">
+      <c r="B70" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="C68" s="11" t="s">
+      <c r="C70" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="D68" s="11" t="s">
+      <c r="D70" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="E68" s="10" t="s">
+      <c r="E70" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="F68" s="12" t="s">
+      <c r="F70" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="G68" s="13" t="s">
+      <c r="G70" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="H68" s="14" t="s">
+      <c r="H70" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="I68" s="14" t="s">
+      <c r="I70" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="J68" s="15" t="s">
+      <c r="J70" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="K68" s="15" t="s">
+      <c r="K70" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="L68" s="13">
-        <v>5034324.1320000002</v>
-      </c>
-      <c r="M68" s="13">
-        <v>3132372.1920000007</v>
-      </c>
-      <c r="N68" s="13">
-        <v>2752296.7048927797</v>
-      </c>
-      <c r="O68" s="16">
-        <v>0.6222031219820553</v>
-      </c>
-    </row>
-    <row r="69" spans="1:15" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="19" t="s">
+      <c r="L70" s="13">
+        <v>5212721.5130000003</v>
+      </c>
+      <c r="M70" s="13">
+        <v>3252416.9690000005</v>
+      </c>
+      <c r="N70" s="13">
+        <v>2864769.1032375996</v>
+      </c>
+      <c r="O70" s="16">
+        <v>0.6239383709428562</v>
+      </c>
+    </row>
+    <row r="71" spans="1:15" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="B69" s="20"/>
-      <c r="C69" s="20"/>
-      <c r="D69" s="20"/>
-      <c r="E69" s="20"/>
-      <c r="F69" s="20"/>
-      <c r="G69" s="20"/>
-      <c r="H69" s="20"/>
-      <c r="I69" s="20"/>
-      <c r="J69" s="20"/>
-      <c r="K69" s="20"/>
-      <c r="L69" s="20"/>
-      <c r="M69" s="20"/>
-      <c r="N69" s="20"/>
-      <c r="O69" s="21"/>
-    </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="O71" s="1"/>
+      <c r="B71" s="20"/>
+      <c r="C71" s="20"/>
+      <c r="D71" s="20"/>
+      <c r="E71" s="20"/>
+      <c r="F71" s="20"/>
+      <c r="G71" s="20"/>
+      <c r="H71" s="20"/>
+      <c r="I71" s="20"/>
+      <c r="J71" s="20"/>
+      <c r="K71" s="20"/>
+      <c r="L71" s="20"/>
+      <c r="M71" s="20"/>
+      <c r="N71" s="20"/>
+      <c r="O71" s="21"/>
+    </row>
+    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O73" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="18">
@@ -3775,7 +3869,7 @@
     <mergeCell ref="G6:G7"/>
     <mergeCell ref="H6:H7"/>
     <mergeCell ref="O6:O7"/>
-    <mergeCell ref="A69:O69"/>
+    <mergeCell ref="A71:O71"/>
     <mergeCell ref="I6:I7"/>
     <mergeCell ref="J6:J7"/>
     <mergeCell ref="K6:K7"/>
@@ -3785,6 +3879,6 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="3.9370078740157501E-2" right="3.9370078740157501E-2" top="3.9370078740157501E-2" bottom="3.9370078740157501E-2" header="0.31496062992126" footer="0.31496062992126"/>
-  <pageSetup paperSize="9" scale="85" fitToHeight="8" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="83" fitToHeight="8" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>